<commit_message>
feat: browse database tables and preview images without leaving site
</commit_message>
<xml_diff>
--- a/documents/demonstrations/jsbsim-catalogue.xlsx
+++ b/documents/demonstrations/jsbsim-catalogue.xlsx
@@ -5471,7 +5471,7 @@
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -8031,7 +8031,7 @@
       <c r="H87" s="2" t="n"/>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -11601,7 +11601,7 @@
       <c r="H170" s="2" t="n"/>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -14877,7 +14877,7 @@
       <c r="H245" s="2" t="n"/>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -20855,7 +20855,7 @@
       <c r="H383" s="2" t="n"/>
       <c r="I383" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J383" s="2" t="inlineStr">
@@ -23901,7 +23901,7 @@
       <c r="H455" s="2" t="n"/>
       <c r="I455" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J455" s="2" t="inlineStr">
@@ -26793,7 +26793,7 @@
       <c r="H522" s="2" t="n"/>
       <c r="I522" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J522" s="2" t="inlineStr">
@@ -30485,7 +30485,7 @@
       <c r="H609" s="2" t="n"/>
       <c r="I609" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J609" s="2" t="inlineStr">
@@ -34445,7 +34445,7 @@
       <c r="H700" s="2" t="n"/>
       <c r="I700" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J700" s="2" t="inlineStr">
@@ -37863,7 +37863,7 @@
       <c r="H780" s="2" t="n"/>
       <c r="I780" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J780" s="2" t="inlineStr">
@@ -40539,7 +40539,7 @@
       <c r="H843" s="2" t="n"/>
       <c r="I843" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J843" s="2" t="inlineStr">
@@ -43463,7 +43463,7 @@
       <c r="H912" s="2" t="n"/>
       <c r="I912" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J912" s="2" t="inlineStr">
@@ -47031,7 +47031,7 @@
       <c r="H996" s="2" t="n"/>
       <c r="I996" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J996" s="2" t="inlineStr">
@@ -52223,7 +52223,7 @@
       <c r="H1119" s="2" t="n"/>
       <c r="I1119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J1119" s="2" t="inlineStr">
@@ -54261,7 +54261,7 @@
       <c r="H1167" s="2" t="n"/>
       <c r="I1167" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J1167" s="2" t="inlineStr">
@@ -55683,7 +55683,7 @@
       <c r="H1201" s="2" t="n"/>
       <c r="I1201" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J1201" s="2" t="inlineStr">
@@ -58849,7 +58849,7 @@
       <c r="H1276" s="2" t="n"/>
       <c r="I1276" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T22:28:57+00:00</t>
+          <t>2026-09-13T15:09:35+00:00</t>
         </is>
       </c>
       <c r="J1276" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: unify demo stages around sources engineering and deliverables
</commit_message>
<xml_diff>
--- a/documents/demonstrations/jsbsim-catalogue.xlsx
+++ b/documents/demonstrations/jsbsim-catalogue.xlsx
@@ -5471,7 +5471,7 @@
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -8031,7 +8031,7 @@
       <c r="H87" s="2" t="n"/>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -11601,7 +11601,7 @@
       <c r="H170" s="2" t="n"/>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -14877,7 +14877,7 @@
       <c r="H245" s="2" t="n"/>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -20855,7 +20855,7 @@
       <c r="H383" s="2" t="n"/>
       <c r="I383" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J383" s="2" t="inlineStr">
@@ -23901,7 +23901,7 @@
       <c r="H455" s="2" t="n"/>
       <c r="I455" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J455" s="2" t="inlineStr">
@@ -26793,7 +26793,7 @@
       <c r="H522" s="2" t="n"/>
       <c r="I522" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J522" s="2" t="inlineStr">
@@ -30485,7 +30485,7 @@
       <c r="H609" s="2" t="n"/>
       <c r="I609" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J609" s="2" t="inlineStr">
@@ -34445,7 +34445,7 @@
       <c r="H700" s="2" t="n"/>
       <c r="I700" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J700" s="2" t="inlineStr">
@@ -37863,7 +37863,7 @@
       <c r="H780" s="2" t="n"/>
       <c r="I780" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J780" s="2" t="inlineStr">
@@ -40539,7 +40539,7 @@
       <c r="H843" s="2" t="n"/>
       <c r="I843" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J843" s="2" t="inlineStr">
@@ -43463,7 +43463,7 @@
       <c r="H912" s="2" t="n"/>
       <c r="I912" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J912" s="2" t="inlineStr">
@@ -47031,7 +47031,7 @@
       <c r="H996" s="2" t="n"/>
       <c r="I996" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J996" s="2" t="inlineStr">
@@ -52223,7 +52223,7 @@
       <c r="H1119" s="2" t="n"/>
       <c r="I1119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J1119" s="2" t="inlineStr">
@@ -54261,7 +54261,7 @@
       <c r="H1167" s="2" t="n"/>
       <c r="I1167" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J1167" s="2" t="inlineStr">
@@ -55683,7 +55683,7 @@
       <c r="H1201" s="2" t="n"/>
       <c r="I1201" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J1201" s="2" t="inlineStr">
@@ -58849,7 +58849,7 @@
       <c r="H1276" s="2" t="n"/>
       <c r="I1276" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T15:09:35+00:00</t>
+          <t>2026-09-13T19:16:53+00:00</t>
         </is>
       </c>
       <c r="J1276" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix: present Odoo XML sources before complementary raw CSV
</commit_message>
<xml_diff>
--- a/documents/demonstrations/jsbsim-catalogue.xlsx
+++ b/documents/demonstrations/jsbsim-catalogue.xlsx
@@ -5471,7 +5471,7 @@
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -8031,7 +8031,7 @@
       <c r="H87" s="2" t="n"/>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -11601,7 +11601,7 @@
       <c r="H170" s="2" t="n"/>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -14877,7 +14877,7 @@
       <c r="H245" s="2" t="n"/>
       <c r="I245" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr">
@@ -20855,7 +20855,7 @@
       <c r="H383" s="2" t="n"/>
       <c r="I383" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J383" s="2" t="inlineStr">
@@ -23901,7 +23901,7 @@
       <c r="H455" s="2" t="n"/>
       <c r="I455" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J455" s="2" t="inlineStr">
@@ -26793,7 +26793,7 @@
       <c r="H522" s="2" t="n"/>
       <c r="I522" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J522" s="2" t="inlineStr">
@@ -30485,7 +30485,7 @@
       <c r="H609" s="2" t="n"/>
       <c r="I609" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J609" s="2" t="inlineStr">
@@ -34445,7 +34445,7 @@
       <c r="H700" s="2" t="n"/>
       <c r="I700" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J700" s="2" t="inlineStr">
@@ -37863,7 +37863,7 @@
       <c r="H780" s="2" t="n"/>
       <c r="I780" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J780" s="2" t="inlineStr">
@@ -40539,7 +40539,7 @@
       <c r="H843" s="2" t="n"/>
       <c r="I843" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J843" s="2" t="inlineStr">
@@ -43463,7 +43463,7 @@
       <c r="H912" s="2" t="n"/>
       <c r="I912" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J912" s="2" t="inlineStr">
@@ -47031,7 +47031,7 @@
       <c r="H996" s="2" t="n"/>
       <c r="I996" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J996" s="2" t="inlineStr">
@@ -52223,7 +52223,7 @@
       <c r="H1119" s="2" t="n"/>
       <c r="I1119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J1119" s="2" t="inlineStr">
@@ -54261,7 +54261,7 @@
       <c r="H1167" s="2" t="n"/>
       <c r="I1167" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J1167" s="2" t="inlineStr">
@@ -55683,7 +55683,7 @@
       <c r="H1201" s="2" t="n"/>
       <c r="I1201" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J1201" s="2" t="inlineStr">
@@ -58849,7 +58849,7 @@
       <c r="H1276" s="2" t="n"/>
       <c r="I1276" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T19:16:53+00:00</t>
+          <t>2026-09-14T00:00:34+00:00</t>
         </is>
       </c>
       <c r="J1276" s="2" t="inlineStr">

</xml_diff>